<commit_message>
Auto update nse_indices_1 outputs
</commit_message>
<xml_diff>
--- a/nse_indices_1_dashboard.xlsx
+++ b/nse_indices_1_dashboard.xlsx
@@ -484,7 +484,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>1.4%</t>
+          <t>1.24%</t>
         </is>
       </c>
     </row>
@@ -611,31 +611,31 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Nifty Midcap 100</t>
+          <t>Nifty Midcap 50</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>1.73</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Nifty Midcap 50</t>
+          <t>Nifty Midcap 150</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>1.71</v>
+        <v>1.08</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Nifty Midcap 150</t>
+          <t>Nifty Midcap 100</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>1.08</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="8">
@@ -782,7 +782,7 @@
         <v>16520.349609375</v>
       </c>
       <c r="G2" s="7" t="n">
-        <v>59115.6015625</v>
+        <v>58180.5</v>
       </c>
       <c r="H2" s="7" t="n">
         <v>21476.25</v>
@@ -11016,7 +11016,7 @@
         <v>1.71</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>1.73</v>
+        <v>0.12</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>1.08</v>
@@ -21262,7 +21262,7 @@
         <v>-1.46</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0</v>
+        <v>-1.58</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>-1.7</v>
@@ -31426,12 +31426,12 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Nifty Midcap 100, Nifty 50, Nifty 100</t>
+          <t>Nifty 50, Nifty 100, Nifty 200</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Nifty Midcap 150, Nifty500 Multicap 50:25:25, Nifty Next 50</t>
+          <t>Nifty Midcap 150, Nifty Midcap 100, Nifty500 Multicap 50:25:25</t>
         </is>
       </c>
     </row>

</xml_diff>